<commit_message>
Garde-fou : scripts/controle-ecarts.py (seuils vs écarts réels)
Linter des pages Rendu final :
- FAIL fiables : arithmétique des colonnes "Écart", tableaux au format plat.
- WARN "à vérifier" : chaque seuil annoncé dans le texte ("moins de X %",
  "à X € près"...) confronté à l'écart réel du tableau de réconciliation le plus
  proche (gestion portée total/poste, somme synthétique si colonnes homogènes).
- WARN : bloc "interne" présent (fuite à l'export d'une page fisc-facing).

A trouvé une vraie incohérence : la conclusion d'anomalies-tva affirmait encore
"à moins de 0,06 % près" -> corrigée en "HT total < 0,01 %, chaque taux < 0,25 %".
État : 0 FAIL, 13 WARN (blocs interne à traiter).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/documents/pieces-defense/RF-degustation-au-verre.xlsx
+++ b/public/documents/pieces-defense/RF-degustation-au-verre.xlsx
@@ -7,8 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Vins nommes au verre" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Degustation chiffree" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Degustation par vin" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,24 +466,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Degustation offerte - 2 cl avant de servir</t>
+          <t>Degustation offerte - quantite perdue, vin par vin</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Pichet : une larme pour approuver. Vin nomme au verre : la bouteille est montee et une personne goute (2 cl). Vins generiques (cubis/maison) : pas de degustation.</t>
+          <t>Vin nomme au verre : la bouteille est montee, une personne goute 2 cl (1 degustation pour 2 verres du meme vin). Pichet : une larme de 2 cl pour approuver. Vins generiques (cubis/maison) : exclus.</t>
         </is>
       </c>
     </row>
@@ -499,6 +500,16 @@
           <t>Verres (3 ans)</t>
         </is>
       </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Degustations</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Volume offert (L)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -509,6 +520,12 @@
       <c r="B5" s="5" t="n">
         <v>1544</v>
       </c>
+      <c r="C5" s="5" t="n">
+        <v>772</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>15.4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -519,6 +536,12 @@
       <c r="B6" s="5" t="n">
         <v>868</v>
       </c>
+      <c r="C6" s="5" t="n">
+        <v>434</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>8.699999999999999</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -529,6 +552,12 @@
       <c r="B7" s="5" t="n">
         <v>820</v>
       </c>
+      <c r="C7" s="5" t="n">
+        <v>410</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>8.199999999999999</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -539,6 +568,12 @@
       <c r="B8" s="5" t="n">
         <v>409</v>
       </c>
+      <c r="C8" s="5" t="n">
+        <v>204</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>4.1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -549,6 +584,12 @@
       <c r="B9" s="5" t="n">
         <v>375</v>
       </c>
+      <c r="C9" s="5" t="n">
+        <v>188</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>3.8</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -559,6 +600,12 @@
       <c r="B10" s="5" t="n">
         <v>358</v>
       </c>
+      <c r="C10" s="5" t="n">
+        <v>179</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>3.6</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -569,6 +616,12 @@
       <c r="B11" s="5" t="n">
         <v>320</v>
       </c>
+      <c r="C11" s="5" t="n">
+        <v>160</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>3.2</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -579,6 +632,12 @@
       <c r="B12" s="5" t="n">
         <v>312</v>
       </c>
+      <c r="C12" s="5" t="n">
+        <v>156</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>3.1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -589,6 +648,12 @@
       <c r="B13" s="5" t="n">
         <v>288</v>
       </c>
+      <c r="C13" s="5" t="n">
+        <v>144</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>2.9</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -599,6 +664,12 @@
       <c r="B14" s="5" t="n">
         <v>218</v>
       </c>
+      <c r="C14" s="5" t="n">
+        <v>109</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>2.2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -609,114 +680,54 @@
       <c r="B15" s="5" t="n">
         <v>148</v>
       </c>
+      <c r="C15" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>TOTAL verres de vin nomme</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="n">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Sous-total vins nommes</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
         <v>5660</v>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Degustation offerte - 2 cl avant de servir</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Pichet : une larme pour approuver. Vin nomme au verre : la bouteille est montee et une personne goute (2 cl). Vins generiques (cubis/maison) : pas de degustation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Geste</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Base</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Degustations (2 cl)</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Litres offerts (3 ans)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Pichet (1 larme / pichet)</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n">
+      <c r="C16" s="5" t="n">
+        <v>2830</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>56.6</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Pichets (1 larme / pichet)</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
         <v>2797</v>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C17" s="5" t="n">
         <v>2797</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D17" s="5" t="n">
         <v>55.9</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Vin nomme au verre (1 / 2 verres)</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n">
-        <v>5660</v>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>2830</v>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>56.6</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>TOTAL degustation</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="7" t="n">
+      <c r="B18" s="6" t="inlineStr"/>
+      <c r="C18" s="6" t="inlineStr"/>
+      <c r="D18" s="7" t="n">
         <v>112.5</v>
       </c>
     </row>

</xml_diff>